<commit_message>
Fig.7 (irregular mix): workload type under each phase name; type column in xlsx; title spacing
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig7_mixT.xlsx
+++ b/figs/data/fig7_mixT.xlsx
@@ -586,7 +586,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>18</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -608,7 +608,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>18</col>
       <colOff>0</colOff>
       <row>22</row>
       <rowOff>0</rowOff>
@@ -630,7 +630,7 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>17</col>
+      <col>18</col>
       <colOff>0</colOff>
       <row>43</row>
       <rowOff>0</rowOff>
@@ -942,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R61"/>
+  <dimension ref="A1:S61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -998,15 +998,20 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>종류</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>시작(h, v4)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>iCAT-v4 (제안)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>CAT-37 (기본값)</t>
         </is>
@@ -1045,13 +1050,18 @@
           <t>YCSB-A</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SQLite DB 읽기50·수정50</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
         <v>-0.002</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>1.025</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>1.027</v>
       </c>
     </row>
@@ -1088,13 +1098,18 @@
           <t>OLTP</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>DB 서버 흉내 (Filebench)</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
         <v>1.118</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>1.121</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>1.179</v>
       </c>
     </row>
@@ -1131,13 +1146,18 @@
           <t>Varmail</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>메일 서버 흉내 (Filebench)</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
         <v>2.25</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>1.611</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>1.929</v>
       </c>
     </row>
@@ -1174,13 +1194,18 @@
           <t>YCSB-A</t>
         </is>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SQLite DB 읽기50·수정50</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
         <v>3.362</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>1.006</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>1.008</v>
       </c>
     </row>
@@ -1217,13 +1242,18 @@
           <t>YCSB-B</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SQLite DB 읽기95·수정5</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
         <v>4.475</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>1.073</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>1.168</v>
       </c>
     </row>
@@ -1260,13 +1290,18 @@
           <t>FIO-Fast</t>
         </is>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>합성 덮어쓰기 (FIO 3영역)</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
         <v>5.591</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>5.574</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>5.706</v>
       </c>
     </row>
@@ -1303,13 +1338,18 @@
           <t>Varmail</t>
         </is>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>메일 서버 흉내 (Filebench)</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
         <v>6.703</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>2.149</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>2.553</v>
       </c>
     </row>
@@ -1346,13 +1386,18 @@
           <t>YCSB-A</t>
         </is>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SQLite DB 읽기50·수정50</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
         <v>7.815</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>1.01</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>1.01</v>
       </c>
     </row>
@@ -1389,13 +1434,18 @@
           <t>OLTP</t>
         </is>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>DB 서버 흉내 (Filebench)</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
         <v>8.930999999999999</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>1.277</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>1.493</v>
       </c>
     </row>
@@ -1429,10 +1479,10 @@
           <t>10시간 전체</t>
         </is>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>2.076</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>2.33</v>
       </c>
     </row>

</xml_diff>